<commit_message>
Acilis guncelleme 2026-10-27 04:50 UTC
</commit_message>
<xml_diff>
--- a/oranlar_yaklasan.xlsx
+++ b/oranlar_yaklasan.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA4"/>
+  <dimension ref="A1:BA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -682,355 +682,6 @@
           <t>Skor</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>4454036</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>02:30</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>BR2</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Juventude</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Nautico</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="H2" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="I2" t="n">
-        <v>5.21</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1.96</v>
-      </c>
-      <c r="M2" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="N2" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="O2" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="P2" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>3.59</v>
-      </c>
-      <c r="R2" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="S2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="T2" t="n">
-        <v>2.01</v>
-      </c>
-      <c r="U2" t="n">
-        <v>5.54</v>
-      </c>
-      <c r="V2" t="n">
-        <v>1.79</v>
-      </c>
-      <c r="W2" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="X2" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>2.39</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>2.85</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>4475907</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ARJ</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Instituto Cord</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Riestra</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>1.79</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2.72</v>
-      </c>
-      <c r="I3" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="K3" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="M3" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="N3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="O3" t="n">
-        <v>1.99</v>
-      </c>
-      <c r="P3" t="n">
-        <v>1.82</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>6.28</v>
-      </c>
-      <c r="R3" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="S3" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="T3" t="n">
-        <v>1.69</v>
-      </c>
-      <c r="U3" t="n">
-        <v>4.88</v>
-      </c>
-      <c r="V3" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="W3" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="X3" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>5.53</v>
-      </c>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>4513960</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>04:05</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>KOL</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Bucaramanga</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="H4" t="n">
-        <v>2.94</v>
-      </c>
-      <c r="I4" t="n">
-        <v>3.53</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1.56</v>
-      </c>
-      <c r="M4" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="N4" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="T4" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="U4" t="n">
-        <v>4.16</v>
-      </c>
-      <c r="V4" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="W4" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="inlineStr"/>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>